<commit_message>
Terminada la primer etapa (listo para entregar)
</commit_message>
<xml_diff>
--- a/Simulación prueba.xlsx
+++ b/Simulación prueba.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27705"/>
   <workbookPr codeName="ThisWorkbook" hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\facun\Documents\Facultad\3er Año\1er Cuatri\Modelos y Simulación\Unidades\U1 Introducción a la Simulación\Práctica\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jhon\Documents\GitHub\Universidad\ProyectoModelo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A0ECAC-3C9D-4867-988E-C1CD62D2F76F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38018730-74CF-426B-BE9B-6392ACE1327D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="E1" sheetId="1" r:id="rId1"/>
-    <sheet name="E2" sheetId="3" r:id="rId2"/>
+    <sheet name="Airport" sheetId="1" r:id="rId1"/>
+    <sheet name="." sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +28,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
@@ -36,8 +35,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="37">
   <si>
     <t>Tiempo entre arribo</t>
   </si>
@@ -45,9 +66,6 @@
     <t>Arribo (Clock)</t>
   </si>
   <si>
-    <t>Duración de Inspección</t>
-  </si>
-  <si>
     <t>P(x)</t>
   </si>
   <si>
@@ -57,18 +75,12 @@
     <t>F</t>
   </si>
   <si>
-    <t>Ocio</t>
-  </si>
-  <si>
     <t>Espera</t>
   </si>
   <si>
     <t>RandomArribo(x)</t>
   </si>
   <si>
-    <t>RandomInspección(x)</t>
-  </si>
-  <si>
     <t>Salida</t>
   </si>
   <si>
@@ -96,9 +108,6 @@
     <t>Tiempo de Facu</t>
   </si>
   <si>
-    <t>Inicio de Inspección (Clock)</t>
-  </si>
-  <si>
     <t>x</t>
   </si>
   <si>
@@ -117,7 +126,49 @@
     <t>Max</t>
   </si>
   <si>
-    <t>Salida (Clock)</t>
+    <t>Spawn (Clock)</t>
+  </si>
+  <si>
+    <t>StartService(Clock)</t>
+  </si>
+  <si>
+    <t>InspDuration</t>
+  </si>
+  <si>
+    <t>Out (Clock)</t>
+  </si>
+  <si>
+    <t>Idle</t>
+  </si>
+  <si>
+    <t>Transit</t>
+  </si>
+  <si>
+    <t>Wait</t>
+  </si>
+  <si>
+    <t>TimeBtwArrival</t>
+  </si>
+  <si>
+    <t>ServiceDuration</t>
+  </si>
+  <si>
+    <t>RandArrival(x)</t>
+  </si>
+  <si>
+    <t>RandService(x)</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Statistic</t>
+  </si>
+  <si>
+    <t>Min</t>
+  </si>
+  <si>
+    <t>Mid</t>
   </si>
 </sst>
 </file>
@@ -159,13 +210,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="10">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -186,22 +262,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41144B02-F783-4812-95E0-751916B51BD0}" name="Table1" displayName="Table1" ref="A1:K13" totalsRowShown="0">
-  <autoFilter ref="A1:K13" xr:uid="{41144B02-F783-4812-95E0-751916B51BD0}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{41144B02-F783-4812-95E0-751916B51BD0}" name="Table1" displayName="Table1" ref="A1:K15" totalsRowShown="0">
+  <autoFilter ref="A1:K15" xr:uid="{41144B02-F783-4812-95E0-751916B51BD0}"/>
   <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{7015C11E-937D-42B0-A90E-4171CEB7DD63}" name="N°"/>
-    <tableColumn id="10" xr3:uid="{B479D487-1331-4FFD-A1D8-D9C8BEB6FB86}" name="RandomArribo(x)"/>
-    <tableColumn id="2" xr3:uid="{1B7A5D8D-4E4D-4940-BD1D-A64A37B690DE}" name="Tiempo entre arribo"/>
-    <tableColumn id="3" xr3:uid="{43F31629-1A66-40C6-AC4F-CAE7D0E1481E}" name="Arribo (Clock)"/>
-    <tableColumn id="4" xr3:uid="{1FB29065-CCF6-499E-85AF-B8DF2EB0ACFC}" name="Inicio de Inspección (Clock)"/>
-    <tableColumn id="12" xr3:uid="{D3CB59A9-ED16-4117-9F8C-C1F36788898F}" name="RandomInspección(x)"/>
-    <tableColumn id="5" xr3:uid="{DB41D0EE-F696-4E42-9FE4-39AF3CB8B233}" name="Duración de Inspección"/>
-    <tableColumn id="13" xr3:uid="{872D993C-AD03-473B-9AE4-BF5B4256B2F2}" name="Salida (Clock)"/>
-    <tableColumn id="7" xr3:uid="{DD6F25BB-7472-4D89-8000-72A8239F69A9}" name="Ocio"/>
-    <tableColumn id="14" xr3:uid="{9C195093-FB81-44F3-942A-9FEB95316607}" name="Transito" dataDxfId="1">
-      <calculatedColumnFormula>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</calculatedColumnFormula>
+    <tableColumn id="10" xr3:uid="{B479D487-1331-4FFD-A1D8-D9C8BEB6FB86}" name="RandArrival(x)"/>
+    <tableColumn id="2" xr3:uid="{1B7A5D8D-4E4D-4940-BD1D-A64A37B690DE}" name="Tiempo entre arribo" dataDxfId="8">
+      <calculatedColumnFormula array="1">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=Table2[[#This Row],[F]],Table2[[#This Row],[TimeBtwArrival]],Table1[[#This Row],[RandArrival(x)]]&lt;=O3,15,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{7D501633-BD8D-4E7A-B9E6-BB79484980F0}" name="Espera"/>
+    <tableColumn id="3" xr3:uid="{43F31629-1A66-40C6-AC4F-CAE7D0E1481E}" name="Spawn (Clock)" dataDxfId="7">
+      <calculatedColumnFormula>SUM(_FV(Table1[[#This Row],[Tiempo entre arribo]],"D2"))</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{1FB29065-CCF6-499E-85AF-B8DF2EB0ACFC}" name="StartService(Clock)" dataDxfId="6">
+      <calculatedColumnFormula>IF(H1&gt;=Table1[[#This Row],[Spawn (Clock)]],H1,Table1[[#This Row],[Spawn (Clock)]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="12" xr3:uid="{D3CB59A9-ED16-4117-9F8C-C1F36788898F}" name="RandService(x)"/>
+    <tableColumn id="5" xr3:uid="{DB41D0EE-F696-4E42-9FE4-39AF3CB8B233}" name="InspDuration" dataDxfId="3">
+      <calculatedColumnFormula array="1">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="13" xr3:uid="{872D993C-AD03-473B-9AE4-BF5B4256B2F2}" name="Out (Clock)" dataDxfId="5">
+      <calculatedColumnFormula>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="7" xr3:uid="{DD6F25BB-7472-4D89-8000-72A8239F69A9}" name="Idle"/>
+    <tableColumn id="14" xr3:uid="{9C195093-FB81-44F3-942A-9FEB95316607}" name="Transit" dataDxfId="4">
+      <calculatedColumnFormula>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{7D501633-BD8D-4E7A-B9E6-BB79484980F0}" name="Wait"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -211,7 +297,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{8289C7F9-5FEA-4CC7-BB9B-7F2E0AF1020C}" name="Table2" displayName="Table2" ref="M1:O4" totalsRowShown="0">
   <autoFilter ref="M1:O4" xr:uid="{8289C7F9-5FEA-4CC7-BB9B-7F2E0AF1020C}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{E7A0C7B7-B4E4-44DC-BF66-CF1B2FB52F9A}" name="Tiempo Entre Arribo"/>
+    <tableColumn id="1" xr3:uid="{E7A0C7B7-B4E4-44DC-BF66-CF1B2FB52F9A}" name="TimeBtwArrival"/>
     <tableColumn id="2" xr3:uid="{5D99FF41-5505-4A75-97DD-E903E8D82892}" name="P(x)"/>
     <tableColumn id="3" xr3:uid="{61835A78-2E9B-4E24-85D9-FDCBD3B752D3}" name="F"/>
   </tableColumns>
@@ -220,10 +306,10 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{43BFA89B-E913-4FC3-A33C-6F6D043CE390}" name="Table3" displayName="Table3" ref="M6:O12" totalsRowShown="0">
-  <autoFilter ref="M6:O12" xr:uid="{43BFA89B-E913-4FC3-A33C-6F6D043CE390}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{43BFA89B-E913-4FC3-A33C-6F6D043CE390}" name="Table3" displayName="Table3" ref="M8:O12" totalsRowShown="0">
+  <autoFilter ref="M8:O12" xr:uid="{43BFA89B-E913-4FC3-A33C-6F6D043CE390}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{49124059-6C29-403B-BB5A-AB77B1667278}" name="Duración de Inspección"/>
+    <tableColumn id="1" xr3:uid="{49124059-6C29-403B-BB5A-AB77B1667278}" name="ServiceDuration"/>
     <tableColumn id="2" xr3:uid="{6386B2A1-CEFD-4318-86EE-D387FFBB18E1}" name="P(x)"/>
     <tableColumn id="3" xr3:uid="{A86BBF1F-79EE-4D99-8045-E78683C1B5FE}" name="F"/>
   </tableColumns>
@@ -232,6 +318,25 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{2C032E18-AD90-42ED-94AB-F28DF8693EDB}" name="Table9" displayName="Table9" ref="H17:K20" totalsRowShown="0">
+  <autoFilter ref="H17:K20" xr:uid="{2C032E18-AD90-42ED-94AB-F28DF8693EDB}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{DE6B4444-23E6-4FDE-B093-0E058C3DF2B6}" name="Statistic"/>
+    <tableColumn id="2" xr3:uid="{DB2F2983-403E-46CC-BF2D-DD39176F7BC6}" name="Wait" dataDxfId="2">
+      <calculatedColumnFormula>MAX(Table1[Wait])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{2E5089C6-5229-4DE1-81AA-1FA9667C8F21}" name="Idle" dataDxfId="1">
+      <calculatedColumnFormula>MAX(Table1[Idle])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="4" xr3:uid="{527FFFE9-5C06-4AB0-A750-3CAF6D141635}" name="Transit" dataDxfId="0">
+      <calculatedColumnFormula>MAX(Table1[Transit])</calculatedColumnFormula>
+    </tableColumn>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B4C43BD3-FE68-41CF-AB96-F973BEA4560E}" name="Table15" displayName="Table15" ref="A1:N27" totalsRowShown="0">
   <autoFilter ref="A1:N27" xr:uid="{41144B02-F783-4812-95E0-751916B51BD0}"/>
   <tableColumns count="14">
@@ -247,7 +352,7 @@
     <tableColumn id="13" xr3:uid="{F5601D7F-47DE-4976-B9C7-F5C9D38DFDEE}" name="Salida"/>
     <tableColumn id="7" xr3:uid="{AE72381E-6C47-4753-BAF8-E2882AB9A0AF}" name="Ocio Juan"/>
     <tableColumn id="12" xr3:uid="{E7818327-4CA5-4A89-B4E6-F7C0E770B365}" name="Ocio Facu"/>
-    <tableColumn id="14" xr3:uid="{45BF0F5B-851C-430E-9CAB-C8B155D3A2D9}" name="Transito" dataDxfId="0">
+    <tableColumn id="14" xr3:uid="{45BF0F5B-851C-430E-9CAB-C8B155D3A2D9}" name="Transito" dataDxfId="9">
       <calculatedColumnFormula>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{81D41C5D-92D1-4DC8-B341-B865B2845198}" name="Espera"/>
@@ -256,7 +361,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C3FACB6E-5C60-4527-9EE3-7D2CA388CA77}" name="Table26" displayName="Table26" ref="P1:R5" totalsRowShown="0">
   <autoFilter ref="P1:R5" xr:uid="{8289C7F9-5FEA-4CC7-BB9B-7F2E0AF1020C}"/>
   <tableColumns count="3">
@@ -268,7 +373,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{6DA988FA-92D7-4AD2-98DF-AA32A27C2C14}" name="Table37" displayName="Table37" ref="P9:R13" totalsRowShown="0">
   <autoFilter ref="P9:R13" xr:uid="{43BFA89B-E913-4FC3-A33C-6F6D043CE390}"/>
   <tableColumns count="3">
@@ -280,7 +385,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{F8A7FA73-10B7-4D3F-9AEF-596931C8CB2E}" name="Table378" displayName="Table378" ref="P17:R21" totalsRowShown="0">
   <autoFilter ref="P17:R21" xr:uid="{F8A7FA73-10B7-4D3F-9AEF-596931C8CB2E}"/>
   <tableColumns count="3">
@@ -556,74 +661,74 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="22.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="23" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="6.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="23" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="11" width="10.42578125" customWidth="1"/>
+    <col min="12" max="12" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.85546875" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="E1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F1" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="G1" t="s">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="H1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" t="s">
         <v>26</v>
       </c>
-      <c r="I1" t="s">
-        <v>6</v>
-      </c>
       <c r="J1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="K1" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="M1" t="s">
+        <v>29</v>
+      </c>
+      <c r="N1" t="s">
+        <v>2</v>
+      </c>
+      <c r="O1" t="s">
         <v>4</v>
       </c>
-      <c r="N1" t="s">
-        <v>3</v>
-      </c>
-      <c r="O1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -635,519 +740,693 @@
         <v>0</v>
       </c>
       <c r="F2">
-        <v>0.88</v>
-      </c>
-      <c r="G2">
-        <v>5</v>
+        <v>0.73</v>
+      </c>
+      <c r="G2" cm="1">
+        <f t="array" ref="G2">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>13</v>
       </c>
       <c r="H2">
-        <v>5</v>
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>13</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>5</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>13</v>
       </c>
       <c r="K2">
         <v>0</v>
       </c>
       <c r="M2">
+        <v>10</v>
+      </c>
+      <c r="N2">
+        <v>0.35</v>
+      </c>
+      <c r="O2">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>0.92</v>
+      </c>
+      <c r="C3" cm="1">
+        <f t="array" ref="C3">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>17</v>
+      </c>
+      <c r="D3">
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D2)</f>
+        <v>17</v>
+      </c>
+      <c r="E3">
+        <f>IF(H2&gt;=Table1[[#This Row],[Spawn (Clock)]],H2,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>17</v>
+      </c>
+      <c r="F3">
+        <v>0.92</v>
+      </c>
+      <c r="G3" cm="1">
+        <f t="array" ref="G3">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>15</v>
+      </c>
+      <c r="H3">
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>32</v>
+      </c>
+      <c r="I3">
+        <f>IF(H2&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H2,0)</f>
         <v>4</v>
       </c>
-      <c r="N2">
-        <v>0.34</v>
-      </c>
-      <c r="O2">
-        <v>0.34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>0.44</v>
-      </c>
-      <c r="C3">
-        <v>5</v>
-      </c>
-      <c r="D3">
-        <v>5</v>
-      </c>
-      <c r="E3">
-        <v>5</v>
-      </c>
-      <c r="F3">
-        <v>0.98</v>
-      </c>
-      <c r="G3">
-        <v>6</v>
-      </c>
-      <c r="H3">
-        <v>11</v>
-      </c>
-      <c r="I3">
-        <v>0</v>
-      </c>
       <c r="J3">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>6</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>15</v>
       </c>
       <c r="K3">
+        <f>IF(H2&gt;Table1[[#This Row],[Spawn (Clock)]],H2-Table1[[#This Row],[Spawn (Clock)]],0)</f>
         <v>0</v>
       </c>
       <c r="M3">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="N3">
-        <v>0.48</v>
+        <v>0.45</v>
       </c>
       <c r="O3">
-        <v>0.82</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>0.64</v>
-      </c>
-      <c r="C4">
-        <v>5</v>
+        <v>0.67</v>
+      </c>
+      <c r="C4" cm="1">
+        <f t="array" ref="C4">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>15</v>
       </c>
       <c r="D4">
-        <v>10</v>
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D3)</f>
+        <v>32</v>
       </c>
       <c r="E4">
-        <v>11</v>
+        <f>IF(H3&gt;=Table1[[#This Row],[Spawn (Clock)]],H3,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>32</v>
       </c>
       <c r="F4">
-        <v>0.99</v>
-      </c>
-      <c r="G4">
-        <v>6</v>
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="G4" cm="1">
+        <f t="array" ref="G4">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>8</v>
       </c>
       <c r="H4">
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>40</v>
+      </c>
+      <c r="I4">
+        <f>IF(H3&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H3,0)</f>
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>8</v>
+      </c>
+      <c r="K4">
+        <f>IF(H3&gt;Table1[[#This Row],[Spawn (Clock)]],H3-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>0</v>
+      </c>
+      <c r="M4">
         <v>17</v>
       </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>7</v>
-      </c>
-      <c r="K4">
-        <v>1</v>
-      </c>
-      <c r="M4">
-        <v>7</v>
-      </c>
       <c r="N4">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="O4">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0.89</v>
-      </c>
-      <c r="C5">
-        <v>7</v>
+        <v>0.02</v>
+      </c>
+      <c r="C5" cm="1">
+        <f t="array" ref="C5">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>10</v>
       </c>
       <c r="D5">
-        <v>17</v>
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D4)</f>
+        <v>42</v>
       </c>
       <c r="E5">
-        <v>17</v>
+        <f>IF(H4&gt;=Table1[[#This Row],[Spawn (Clock)]],H4,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>42</v>
       </c>
       <c r="F5">
-        <v>0.15</v>
-      </c>
-      <c r="G5">
-        <v>2</v>
+        <v>0.97</v>
+      </c>
+      <c r="G5" cm="1">
+        <f t="array" ref="G5">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>15</v>
       </c>
       <c r="H5">
-        <v>19</v>
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>57</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <f>IF(H4&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H4,0)</f>
+        <v>2</v>
       </c>
       <c r="J5">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>2</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>15</v>
       </c>
       <c r="K5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+        <f>IF(H4&gt;Table1[[#This Row],[Spawn (Clock)]],H4-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
-        <v>0.65</v>
-      </c>
-      <c r="C6">
-        <v>5</v>
+        <v>0.80500000000000005</v>
+      </c>
+      <c r="C6" cm="1">
+        <f t="array" ref="C6">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>17</v>
       </c>
       <c r="D6">
-        <v>22</v>
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D5)</f>
+        <v>59</v>
       </c>
       <c r="E6">
-        <v>22</v>
+        <f>IF(H5&gt;=Table1[[#This Row],[Spawn (Clock)]],H5,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>59</v>
       </c>
       <c r="F6">
-        <v>0.6</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
+        <v>0.15</v>
+      </c>
+      <c r="G6" cm="1">
+        <f t="array" ref="G6">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>8</v>
       </c>
       <c r="H6">
-        <v>26</v>
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>67</v>
       </c>
       <c r="I6">
-        <v>3</v>
+        <f>IF(H5&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H5,0)</f>
+        <v>2</v>
       </c>
       <c r="J6">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>4</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>8</v>
       </c>
       <c r="K6">
-        <v>0</v>
-      </c>
-      <c r="M6" t="s">
-        <v>2</v>
-      </c>
-      <c r="N6" t="s">
-        <v>3</v>
-      </c>
-      <c r="O6" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+        <f>IF(H5&gt;Table1[[#This Row],[Spawn (Clock)]],H5-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>0.7</v>
-      </c>
-      <c r="C7">
-        <v>5</v>
+        <v>0.92</v>
+      </c>
+      <c r="C7" cm="1">
+        <f t="array" ref="C7">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>17</v>
       </c>
       <c r="D7">
-        <v>27</v>
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D6)</f>
+        <v>76</v>
       </c>
       <c r="E7">
-        <v>27</v>
+        <f>IF(H6&gt;=Table1[[#This Row],[Spawn (Clock)]],H6,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>76</v>
       </c>
       <c r="F7">
-        <v>0.65</v>
-      </c>
-      <c r="G7">
-        <v>4</v>
+        <v>0.76</v>
+      </c>
+      <c r="G7" cm="1">
+        <f t="array" ref="G7">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>13</v>
       </c>
       <c r="H7">
-        <v>31</v>
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>89</v>
       </c>
       <c r="I7">
-        <v>1</v>
+        <f>IF(H6&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H6,0)</f>
+        <v>9</v>
       </c>
       <c r="J7">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>4</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>13</v>
       </c>
       <c r="K7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>1</v>
-      </c>
-      <c r="N7">
-        <v>0.05</v>
-      </c>
-      <c r="O7">
-        <v>0.05</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+        <f>IF(H6&gt;Table1[[#This Row],[Spawn (Clock)]],H6-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
-        <v>0.44</v>
-      </c>
-      <c r="C8">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="C8" cm="1">
+        <f t="array" ref="C8">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>10</v>
       </c>
       <c r="D8">
-        <v>32</v>
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D7)</f>
+        <v>86</v>
       </c>
       <c r="E8">
-        <v>32</v>
+        <f>IF(H7&gt;=Table1[[#This Row],[Spawn (Clock)]],H7,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>89</v>
       </c>
       <c r="F8">
-        <v>0.82</v>
-      </c>
-      <c r="G8">
-        <v>5</v>
+        <v>0.96</v>
+      </c>
+      <c r="G8" cm="1">
+        <f t="array" ref="G8">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>15</v>
       </c>
       <c r="H8">
-        <v>37</v>
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>104</v>
       </c>
       <c r="I8">
-        <v>1</v>
+        <f>IF(H7&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H7,0)</f>
+        <v>0</v>
       </c>
       <c r="J8">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>5</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>18</v>
       </c>
       <c r="K8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>2</v>
-      </c>
-      <c r="N8">
-        <v>0.17</v>
-      </c>
-      <c r="O8">
-        <v>0.22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+        <f>IF(H7&gt;Table1[[#This Row],[Spawn (Clock)]],H7-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>3</v>
+      </c>
+      <c r="M8" t="s">
+        <v>30</v>
+      </c>
+      <c r="N8" t="s">
+        <v>2</v>
+      </c>
+      <c r="O8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>0.53</v>
-      </c>
-      <c r="C9">
-        <v>5</v>
+        <v>0.73</v>
+      </c>
+      <c r="C9" cm="1">
+        <f t="array" ref="C9">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>15</v>
       </c>
       <c r="D9">
-        <v>37</v>
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D8)</f>
+        <v>101</v>
       </c>
       <c r="E9">
-        <v>37</v>
+        <f>IF(H8&gt;=Table1[[#This Row],[Spawn (Clock)]],H8,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>104</v>
       </c>
       <c r="F9">
-        <v>0.96</v>
-      </c>
-      <c r="G9">
-        <v>6</v>
+        <v>0.19</v>
+      </c>
+      <c r="G9" cm="1">
+        <f t="array" ref="G9">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>8</v>
       </c>
       <c r="H9">
-        <v>43</v>
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>112</v>
       </c>
       <c r="I9">
+        <f>IF(H8&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H8,0)</f>
         <v>0</v>
       </c>
       <c r="J9">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>6</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>11</v>
       </c>
       <c r="K9">
-        <v>0</v>
+        <f>IF(H8&gt;Table1[[#This Row],[Spawn (Clock)]],H8-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>3</v>
       </c>
       <c r="M9">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="N9">
-        <v>0.23</v>
+        <v>0.38</v>
       </c>
       <c r="O9">
-        <v>0.45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
-        <v>0.77</v>
-      </c>
-      <c r="C10">
-        <v>5</v>
+        <v>0.82</v>
+      </c>
+      <c r="C10" cm="1">
+        <f t="array" ref="C10">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>17</v>
       </c>
       <c r="D10">
-        <v>42</v>
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D9)</f>
+        <v>118</v>
       </c>
       <c r="E10">
-        <v>43</v>
+        <f>IF(H9&gt;=Table1[[#This Row],[Spawn (Clock)]],H9,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>118</v>
       </c>
       <c r="F10">
-        <v>0.82</v>
-      </c>
-      <c r="G10">
-        <v>5</v>
+        <v>0.33</v>
+      </c>
+      <c r="G10" cm="1">
+        <f t="array" ref="G10">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>8</v>
       </c>
       <c r="H10">
-        <v>48</v>
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>126</v>
       </c>
       <c r="I10">
-        <v>0</v>
+        <f>IF(H9&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H9,0)</f>
+        <v>6</v>
       </c>
       <c r="J10">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>6</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>8</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <f>IF(H9&gt;Table1[[#This Row],[Spawn (Clock)]],H9-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>0</v>
       </c>
       <c r="M10">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="N10">
-        <v>0.25</v>
+        <v>0.32</v>
       </c>
       <c r="O10">
         <v>0.7</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
-        <v>0.76</v>
-      </c>
-      <c r="C11">
-        <v>5</v>
+        <v>0.75</v>
+      </c>
+      <c r="C11" cm="1">
+        <f t="array" ref="C11">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>15</v>
       </c>
       <c r="D11">
-        <v>47</v>
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D10)</f>
+        <v>133</v>
       </c>
       <c r="E11">
-        <v>48</v>
-      </c>
-      <c r="F11">
-        <v>0.67</v>
-      </c>
-      <c r="G11">
-        <v>4</v>
+        <f>IF(H10&gt;=Table1[[#This Row],[Spawn (Clock)]],H10,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>133</v>
+      </c>
+      <c r="G11" cm="1">
+        <f t="array" ref="G11">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>8</v>
       </c>
       <c r="H11">
-        <v>52</v>
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>141</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <f>IF(H10&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H10,0)</f>
+        <v>7</v>
       </c>
       <c r="J11">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>5</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>8</v>
       </c>
       <c r="K11">
-        <v>1</v>
+        <f>IF(H10&gt;Table1[[#This Row],[Spawn (Clock)]],H10-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>0</v>
       </c>
       <c r="M11">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="N11">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="O11">
-        <v>0.88</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
-      <c r="B12">
-        <v>0.54</v>
-      </c>
-      <c r="C12">
-        <v>5</v>
+      <c r="C12" cm="1">
+        <f t="array" ref="C12">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>10</v>
       </c>
       <c r="D12">
-        <v>52</v>
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D11)</f>
+        <v>143</v>
       </c>
       <c r="E12">
-        <v>52</v>
-      </c>
-      <c r="F12">
-        <v>0.96</v>
-      </c>
-      <c r="G12">
-        <v>6</v>
+        <f>IF(H11&gt;=Table1[[#This Row],[Spawn (Clock)]],H11,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>143</v>
+      </c>
+      <c r="G12" cm="1">
+        <f t="array" ref="G12">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>8</v>
       </c>
       <c r="H12">
-        <v>58</v>
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>151</v>
       </c>
       <c r="I12">
-        <v>0</v>
+        <f>IF(H11&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H11,0)</f>
+        <v>2</v>
       </c>
       <c r="J12">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>6</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>8</v>
       </c>
       <c r="K12">
+        <f>IF(H11&gt;Table1[[#This Row],[Spawn (Clock)]],H11-Table1[[#This Row],[Spawn (Clock)]],0)</f>
         <v>0</v>
       </c>
       <c r="M12">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="N12">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="O12">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
-      <c r="B13">
-        <v>0.08</v>
-      </c>
-      <c r="C13">
-        <v>4</v>
+      <c r="C13" cm="1">
+        <f t="array" ref="C13">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>10</v>
       </c>
       <c r="D13">
-        <v>56</v>
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D12)</f>
+        <v>153</v>
       </c>
       <c r="E13">
-        <v>58</v>
-      </c>
-      <c r="F13">
-        <v>0.74</v>
-      </c>
-      <c r="G13">
-        <v>5</v>
+        <f>IF(H12&gt;=Table1[[#This Row],[Spawn (Clock)]],H12,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>153</v>
+      </c>
+      <c r="G13" cm="1">
+        <f t="array" ref="G13">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>8</v>
       </c>
       <c r="H13">
-        <v>63</v>
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>161</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <f>IF(H12&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H12,0)</f>
+        <v>2</v>
       </c>
       <c r="J13">
-        <f>SUM(Table1[[#This Row],[Salida (Clock)]],-Table1[[#This Row],[Arribo (Clock)]])</f>
-        <v>7</v>
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>8</v>
       </c>
       <c r="K13">
-        <v>2</v>
+        <f>IF(H12&gt;Table1[[#This Row],[Spawn (Clock)]],H12-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="C14" cm="1">
+        <f t="array" ref="C14">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>10</v>
+      </c>
+      <c r="D14">
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D13)</f>
+        <v>163</v>
+      </c>
+      <c r="E14">
+        <f>IF(H13&gt;=Table1[[#This Row],[Spawn (Clock)]],H13,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>163</v>
+      </c>
+      <c r="G14" cm="1">
+        <f t="array" ref="G14">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>8</v>
+      </c>
+      <c r="H14">
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>171</v>
+      </c>
+      <c r="I14">
+        <f>IF(H13&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H13,0)</f>
+        <v>2</v>
+      </c>
+      <c r="J14" s="1">
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>8</v>
+      </c>
+      <c r="K14">
+        <f>IF(H13&gt;Table1[[#This Row],[Spawn (Clock)]],H13-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="C15" cm="1">
+        <f t="array" ref="C15">_xlfn.IFS(Table1[[#This Row],[RandArrival(x)]]&lt;=O2,M2,Table1[[#This Row],[RandArrival(x)]]&lt;=O3,M3,Table1[[#This Row],[RandArrival(x)]]&lt;=O4,M4)</f>
+        <v>10</v>
+      </c>
+      <c r="D15">
+        <f>SUM(Table1[[#This Row],[Tiempo entre arribo]],D14)</f>
+        <v>173</v>
+      </c>
+      <c r="E15">
+        <f>IF(H14&gt;=Table1[[#This Row],[Spawn (Clock)]],H14,Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>173</v>
+      </c>
+      <c r="G15" cm="1">
+        <f t="array" ref="G15">_xlfn.IFS(Table1[[#This Row],[RandService(x)]]&lt;=O9,M9,Table1[[#This Row],[RandService(x)]]&lt;=O10,M10,Table1[[#This Row],[RandService(x)]]&lt;=O11,M11,Table1[[#This Row],[RandService(x)]]&lt;=O12,M12)</f>
+        <v>8</v>
+      </c>
+      <c r="H15">
+        <f>SUM(Table1[[#This Row],[InspDuration]],Table1[[#This Row],[StartService(Clock)]])</f>
+        <v>181</v>
+      </c>
+      <c r="I15">
+        <f>IF(H14&lt;Table1[[#This Row],[Spawn (Clock)]],Table1[[#This Row],[Spawn (Clock)]]-H14,0)</f>
+        <v>2</v>
+      </c>
+      <c r="J15" s="1">
+        <f>SUM(Table1[[#This Row],[Out (Clock)]],-Table1[[#This Row],[Spawn (Clock)]])</f>
+        <v>8</v>
+      </c>
+      <c r="K15">
+        <f>IF(H14&gt;Table1[[#This Row],[Spawn (Clock)]],H14-Table1[[#This Row],[Spawn (Clock)]],0)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H17" t="s">
+        <v>34</v>
+      </c>
+      <c r="I17" t="s">
+        <v>28</v>
+      </c>
+      <c r="J17" t="s">
+        <v>26</v>
+      </c>
+      <c r="K17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H18" t="s">
+        <v>21</v>
+      </c>
+      <c r="I18">
+        <f>MAX(Table1[Wait])</f>
+        <v>3</v>
+      </c>
+      <c r="J18">
+        <f>MAX(Table1[Idle])</f>
+        <v>9</v>
+      </c>
+      <c r="K18">
+        <f>MAX(Table1[Transit])</f>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H19" t="s">
+        <v>35</v>
+      </c>
+      <c r="I19">
+        <f>MIN(Table1[Wait])</f>
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <f>MIN(Table1[Idle])</f>
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <f>MIN(Table1[Transit])</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="8:11" x14ac:dyDescent="0.25">
+      <c r="H20" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-  <tableParts count="3">
+  <tableParts count="4">
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1156,81 +1435,81 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0C9099E-E3D4-4CC2-AC26-294D124FA050}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:R27"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="29.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="28.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="17" width="23" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
       </c>
       <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" t="s">
+        <v>12</v>
+      </c>
+      <c r="I1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" t="s">
-        <v>14</v>
-      </c>
-      <c r="G1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H1" t="s">
-        <v>15</v>
-      </c>
-      <c r="I1" t="s">
-        <v>16</v>
-      </c>
       <c r="J1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="K1" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="L1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="M1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="N1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="P1" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>2</v>
+      </c>
+      <c r="R1" t="s">
         <v>4</v>
       </c>
-      <c r="Q1" t="s">
-        <v>3</v>
-      </c>
-      <c r="R1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1242,7 +1521,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G2">
         <v>0.5</v>
@@ -1257,7 +1536,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M2">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -1276,7 +1555,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1290,7 +1569,7 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F3">
         <v>2</v>
@@ -1299,7 +1578,7 @@
         <v>0.71</v>
       </c>
       <c r="H3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I3">
         <v>5</v>
@@ -1308,7 +1587,7 @@
         <v>7</v>
       </c>
       <c r="K3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L3">
         <v>2</v>
@@ -1330,7 +1609,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1347,7 +1626,7 @@
         <v>5</v>
       </c>
       <c r="F4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G4">
         <v>0.89</v>
@@ -1356,7 +1635,7 @@
         <v>5</v>
       </c>
       <c r="I4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J4">
         <v>10</v>
@@ -1365,7 +1644,7 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M4">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -1384,7 +1663,7 @@
         <v>0.85</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1398,7 +1677,7 @@
         <v>6</v>
       </c>
       <c r="E5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F5">
         <v>7</v>
@@ -1407,7 +1686,7 @@
         <v>0.19</v>
       </c>
       <c r="H5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I5">
         <v>3</v>
@@ -1416,7 +1695,7 @@
         <v>10</v>
       </c>
       <c r="K5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L5">
         <v>0</v>
@@ -1438,7 +1717,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1455,7 +1734,7 @@
         <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G6">
         <v>0.28000000000000003</v>
@@ -1464,7 +1743,7 @@
         <v>2</v>
       </c>
       <c r="I6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J6">
         <v>12</v>
@@ -1473,7 +1752,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M6">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -1483,7 +1762,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1497,7 +1776,7 @@
         <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F7">
         <v>10</v>
@@ -1506,7 +1785,7 @@
         <v>0.86</v>
       </c>
       <c r="H7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I7">
         <v>6</v>
@@ -1515,7 +1794,7 @@
         <v>16</v>
       </c>
       <c r="K7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L7">
         <v>0</v>
@@ -1528,7 +1807,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1545,7 +1824,7 @@
         <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G8">
         <v>0.55000000000000004</v>
@@ -1554,7 +1833,7 @@
         <v>3</v>
       </c>
       <c r="I8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J8">
         <v>15</v>
@@ -1563,7 +1842,7 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M8">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -1573,7 +1852,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1590,7 +1869,7 @@
         <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G9">
         <v>0.23</v>
@@ -1599,7 +1878,7 @@
         <v>2</v>
       </c>
       <c r="I9" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J9">
         <v>17</v>
@@ -1608,7 +1887,7 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M9">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -1618,16 +1897,16 @@
         <v>2</v>
       </c>
       <c r="P9" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="Q9" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R9" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1644,7 +1923,7 @@
         <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G10">
         <v>0.18</v>
@@ -1653,7 +1932,7 @@
         <v>2</v>
       </c>
       <c r="I10" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J10">
         <v>19</v>
@@ -1662,7 +1941,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M10">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -1681,7 +1960,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1698,7 +1977,7 @@
         <v>19</v>
       </c>
       <c r="F11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G11">
         <v>0.85</v>
@@ -1707,7 +1986,7 @@
         <v>5</v>
       </c>
       <c r="I11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J11">
         <v>24</v>
@@ -1716,7 +1995,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M11">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -1735,7 +2014,7 @@
         <v>0.57999999999999996</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1749,7 +2028,7 @@
         <v>21</v>
       </c>
       <c r="E12" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F12">
         <v>21</v>
@@ -1758,7 +2037,7 @@
         <v>0.39</v>
       </c>
       <c r="H12" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I12">
         <v>4</v>
@@ -1767,7 +2046,7 @@
         <v>25</v>
       </c>
       <c r="K12" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L12">
         <v>5</v>
@@ -1789,7 +2068,7 @@
         <v>0.83</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1806,7 +2085,7 @@
         <v>24</v>
       </c>
       <c r="F13" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G13">
         <v>0.93</v>
@@ -1815,7 +2094,7 @@
         <v>5</v>
       </c>
       <c r="I13" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J13">
         <v>29</v>
@@ -1824,7 +2103,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M13">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -1843,7 +2122,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1857,7 +2136,7 @@
         <v>26</v>
       </c>
       <c r="E14" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F14">
         <v>26</v>
@@ -1866,7 +2145,7 @@
         <v>0.7</v>
       </c>
       <c r="H14" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I14">
         <v>5</v>
@@ -1875,7 +2154,7 @@
         <v>31</v>
       </c>
       <c r="K14" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L14">
         <v>1</v>
@@ -1885,7 +2164,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1902,7 +2181,7 @@
         <v>29</v>
       </c>
       <c r="F15" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G15">
         <v>0.43</v>
@@ -1911,7 +2190,7 @@
         <v>3</v>
       </c>
       <c r="I15" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J15">
         <v>32</v>
@@ -1920,7 +2199,7 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M15">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -1930,7 +2209,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1947,7 +2226,7 @@
         <v>33</v>
       </c>
       <c r="F16" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G16">
         <v>0.35</v>
@@ -1956,7 +2235,7 @@
         <v>3</v>
       </c>
       <c r="I16" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J16">
         <v>36</v>
@@ -1965,7 +2244,7 @@
         <v>1</v>
       </c>
       <c r="L16" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M16">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -1975,7 +2254,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1989,7 +2268,7 @@
         <v>35</v>
       </c>
       <c r="E17" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F17">
         <v>35</v>
@@ -1998,7 +2277,7 @@
         <v>0.37</v>
       </c>
       <c r="H17" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I17">
         <v>4</v>
@@ -2007,7 +2286,7 @@
         <v>39</v>
       </c>
       <c r="K17" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L17">
         <v>4</v>
@@ -2020,16 +2299,16 @@
         <v>0</v>
       </c>
       <c r="P17" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="Q17" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R17" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2046,7 +2325,7 @@
         <v>37</v>
       </c>
       <c r="F18" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G18">
         <v>0.96</v>
@@ -2055,7 +2334,7 @@
         <v>5</v>
       </c>
       <c r="I18" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J18">
         <v>42</v>
@@ -2064,7 +2343,7 @@
         <v>1</v>
       </c>
       <c r="L18" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M18">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -2083,7 +2362,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2097,7 +2376,7 @@
         <v>41</v>
       </c>
       <c r="E19" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F19">
         <v>41</v>
@@ -2106,7 +2385,7 @@
         <v>0.63</v>
       </c>
       <c r="H19" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I19">
         <v>5</v>
@@ -2115,7 +2394,7 @@
         <v>46</v>
       </c>
       <c r="K19" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L19">
         <v>2</v>
@@ -2137,7 +2416,7 @@
         <v>0.62</v>
       </c>
     </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2154,7 +2433,7 @@
         <v>43</v>
       </c>
       <c r="F20" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G20">
         <v>0.56000000000000005</v>
@@ -2163,7 +2442,7 @@
         <v>3</v>
       </c>
       <c r="I20" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J20">
         <v>46</v>
@@ -2172,7 +2451,7 @@
         <v>1</v>
       </c>
       <c r="L20" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M20">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -2191,7 +2470,7 @@
         <v>0.77</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2208,7 +2487,7 @@
         <v>46</v>
       </c>
       <c r="F21" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G21">
         <v>0.78</v>
@@ -2217,7 +2496,7 @@
         <v>4</v>
       </c>
       <c r="I21" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J21">
         <v>50</v>
@@ -2226,7 +2505,7 @@
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M21">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -2245,7 +2524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2262,7 +2541,7 @@
         <v>50</v>
       </c>
       <c r="F22" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G22">
         <v>0.78</v>
@@ -2271,7 +2550,7 @@
         <v>4</v>
       </c>
       <c r="I22" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J22">
         <v>54</v>
@@ -2280,7 +2559,7 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M22">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -2290,7 +2569,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2304,13 +2583,13 @@
         <v>52</v>
       </c>
       <c r="E23" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G23">
         <v>0.88</v>
       </c>
       <c r="H23" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I23">
         <v>6</v>
@@ -2319,7 +2598,7 @@
         <v>58</v>
       </c>
       <c r="K23" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L23">
         <v>6</v>
@@ -2332,7 +2611,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2349,7 +2628,7 @@
         <v>55</v>
       </c>
       <c r="F24" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G24">
         <v>0.84</v>
@@ -2358,7 +2637,7 @@
         <v>5</v>
       </c>
       <c r="I24" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J24">
         <v>60</v>
@@ -2367,7 +2646,7 @@
         <v>1</v>
       </c>
       <c r="L24" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M24">
         <f>SUM(Table15[[#This Row],[Salida]],-Table15[[#This Row],[Arribo (Clock)]])</f>
@@ -2377,7 +2656,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2391,7 +2670,7 @@
         <v>57</v>
       </c>
       <c r="E25" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F25">
         <v>58</v>
@@ -2400,7 +2679,7 @@
         <v>0.93</v>
       </c>
       <c r="H25" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I25">
         <v>6</v>
@@ -2409,7 +2688,7 @@
         <v>64</v>
       </c>
       <c r="K25" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="L25">
         <v>0</v>
@@ -2422,7 +2701,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K26">
         <f>SUM(K2:K25)</f>
         <v>4</v>
@@ -2440,10 +2719,10 @@
         <v>8</v>
       </c>
       <c r="O26" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="L27">
         <f>MAX(L2:L25)</f>
         <v>6</v>
@@ -2457,7 +2736,7 @@
         <v>3</v>
       </c>
       <c r="O27" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>